<commit_message>
added: - test_generate_hmo_billing_reports() a handler so HTTP GET call could trigger the generation. - in hmo_billing.rs, functions to generate HMO billing reports - in report_generation.rs,added_framework for running tokio task. - billing_templates/HMO_Billing_Template.xlsx as the template
</commit_message>
<xml_diff>
--- a/dnc_backend/billing_templates/HMO_Billing_Template.xlsx
+++ b/dnc_backend/billing_templates/HMO_Billing_Template.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="37">
   <si>
     <t xml:space="preserve">                 DENTAL NETWORK COMPANY</t>
   </si>
@@ -99,24 +99,6 @@
   <si>
     <t>Total Amount Due
 (inclusive of 12% VAT)</t>
-  </si>
-  <si>
-    <t>09-12-25N2</t>
-  </si>
-  <si>
-    <t>A2G PROFEC ENGINEERING SERVICES</t>
-  </si>
-  <si>
-    <t>80-12-00209</t>
-  </si>
-  <si>
-    <t>Annually</t>
-  </si>
-  <si>
-    <t>Basic (+) 2 teeth of LC (+) Desensitization of Hypersensitive Teeth (2)</t>
-  </si>
-  <si>
-    <t>9/15/2025 - 9/14/2026</t>
   </si>
   <si>
     <t>paid</t>
@@ -565,7 +547,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="2" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -574,7 +556,7 @@
     <xf numFmtId="49" fontId="7" fillId="2" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="2" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -683,7 +665,7 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>223554</xdr:colOff>
+      <xdr:colOff>223553</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>168088</xdr:rowOff>
     </xdr:from>
@@ -691,7 +673,7 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>1239089</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>61072</xdr:rowOff>
+      <xdr:rowOff>61071</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -710,8 +692,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm flipH="1" rot="10800000">
-          <a:off x="2395254" y="5759263"/>
-          <a:ext cx="1015536" cy="654985"/>
+          <a:off x="2395253" y="5759263"/>
+          <a:ext cx="1015537" cy="654984"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -730,13 +712,13 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>152399</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>190499</xdr:rowOff>
+      <xdr:rowOff>190498</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>333375</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>333374</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -756,8 +738,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="990599" y="190499"/>
-          <a:ext cx="1514477" cy="1000127"/>
+          <a:off x="990599" y="190498"/>
+          <a:ext cx="1514476" cy="1000127"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -827,7 +809,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>2088543</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>161924</xdr:rowOff>
+      <xdr:rowOff>161923</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -847,7 +829,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8271833" y="5870971"/>
-          <a:ext cx="1500211" cy="453629"/>
+          <a:ext cx="1500211" cy="453628"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2260,47 +2242,29 @@
     </row>
     <row r="17" ht="34.5" customHeight="1">
       <c r="A17" s="25"/>
-      <c r="B17" s="30">
-        <v>2</v>
-      </c>
-      <c r="C17" t="s" s="31">
-        <v>21</v>
-      </c>
-      <c r="D17" t="s" s="31">
-        <v>22</v>
-      </c>
-      <c r="E17" t="s" s="32">
-        <v>23</v>
-      </c>
-      <c r="F17" s="33">
-        <v>5</v>
-      </c>
-      <c r="G17" t="s" s="32">
-        <v>24</v>
-      </c>
-      <c r="H17" t="s" s="34">
-        <v>25</v>
-      </c>
-      <c r="I17" t="s" s="34">
-        <v>26</v>
-      </c>
-      <c r="J17" s="35">
-        <v>200</v>
-      </c>
+      <c r="B17" s="30"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
+      <c r="J17" s="35"/>
       <c r="K17" s="35" cm="1">
         <f t="array" ref="K17">J17*0.12</f>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="L17" s="35" cm="1">
         <f t="array" ref="L17">SUM(J17:K17)</f>
-        <v>224</v>
+        <v>0</v>
       </c>
       <c r="M17" s="36" cm="1">
         <f t="array" ref="M17">SUM(F17*L17)</f>
-        <v>1120</v>
+        <v>0</v>
       </c>
       <c r="N17" t="s" s="37">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="O17" s="38"/>
       <c r="P17" s="38"/>
@@ -2309,33 +2273,33 @@
     <row r="18" ht="56.25" customHeight="1">
       <c r="A18" s="25"/>
       <c r="B18" t="s" s="39">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C18" s="40"/>
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
       <c r="F18" s="41" cm="1">
         <f t="array" ref="F18">SUM(F17:F17)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G18" s="42"/>
       <c r="H18" s="42"/>
       <c r="I18" s="42"/>
       <c r="J18" s="43" cm="1">
         <f t="array" ref="J18">SUM(J17:J17)</f>
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="K18" s="43" cm="1">
         <f t="array" ref="K18">SUM(K17:K17)</f>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="L18" s="43" cm="1">
         <f t="array" ref="L18">SUM(L17:L17)</f>
-        <v>224</v>
+        <v>0</v>
       </c>
       <c r="M18" s="43" cm="1">
         <f t="array" ref="M18">SUM(M17:M17)</f>
-        <v>1120</v>
+        <v>0</v>
       </c>
       <c r="N18" s="29"/>
       <c r="O18" s="2"/>
@@ -2384,16 +2348,16 @@
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" t="s" s="47">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D21" s="48"/>
       <c r="E21" t="s" s="49">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" t="s" s="49">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I21" s="50"/>
       <c r="J21" s="2"/>
@@ -2409,7 +2373,7 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" t="s" s="49">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D22" s="50"/>
       <c r="E22" s="50"/>
@@ -2450,10 +2414,10 @@
       <c r="B24" s="2"/>
       <c r="C24" s="50"/>
       <c r="D24" t="s" s="49">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E24" t="s" s="49">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -2472,16 +2436,16 @@
       <c r="A25" s="2"/>
       <c r="B25" s="14"/>
       <c r="C25" t="s" s="52">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D25" s="53"/>
       <c r="E25" t="s" s="49">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" t="s" s="54">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="I25" s="55"/>
       <c r="J25" s="2"/>
@@ -2497,16 +2461,16 @@
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" t="s" s="47">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D26" s="48"/>
       <c r="E26" t="s" s="49">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" t="s" s="49">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="I26" s="50"/>
       <c r="J26" s="2"/>
@@ -2578,7 +2542,7 @@
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2"/>
       <c r="B30" t="s" s="56">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -2599,7 +2563,7 @@
     <row r="31" ht="89.1" customHeight="1">
       <c r="A31" s="2"/>
       <c r="B31" t="s" s="57">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C31" s="58"/>
       <c r="D31" s="58"/>

</xml_diff>